<commit_message>
finished leaflet set up
</commit_message>
<xml_diff>
--- a/Data/Raw_Data/Soil_health_Thresholds.xlsx
+++ b/Data/Raw_Data/Soil_health_Thresholds.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qxnq723\Desktop\Project_2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qxnq723\Desktop\Project_2\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB75175-E619-4F85-9D3D-60D81C65434C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{996CEF6C-AA35-4B99-A4D6-B57863EB365A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9570" yWindow="0" windowWidth="9790" windowHeight="11370" xr2:uid="{ED39DD28-1322-43F7-985E-A196497B6654}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{ED39DD28-1322-43F7-985E-A196497B6654}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="32">
   <si>
     <t>Soil_Metric</t>
   </si>
@@ -108,6 +108,33 @@
   </si>
   <si>
     <t>SVG_threshold</t>
+  </si>
+  <si>
+    <t>HM_name</t>
+  </si>
+  <si>
+    <t>Nickel</t>
+  </si>
+  <si>
+    <t>Arsenic</t>
+  </si>
+  <si>
+    <t>Lead</t>
+  </si>
+  <si>
+    <t>Zirconium</t>
+  </si>
+  <si>
+    <t>Selenium</t>
+  </si>
+  <si>
+    <t>Copper</t>
+  </si>
+  <si>
+    <t>Cadmium</t>
+  </si>
+  <si>
+    <t>Phosphorus</t>
   </si>
 </sst>
 </file>
@@ -479,19 +506,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BD7DD56-4B10-4485-B77C-894712A5E9AA}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.453125" customWidth="1"/>
-    <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="4" max="4" width="13.6328125" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="14.54296875" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" customWidth="1"/>
-    <col min="8" max="8" width="12.7265625" customWidth="1"/>
+    <col min="2" max="3" width="11" customWidth="1"/>
+    <col min="5" max="5" width="13.6328125" customWidth="1"/>
+    <col min="6" max="6" width="16" customWidth="1"/>
+    <col min="7" max="7" width="14.54296875" customWidth="1"/>
+    <col min="8" max="8" width="13.7265625" customWidth="1"/>
+    <col min="9" max="9" width="12.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -499,36 +526,39 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>18</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>22</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>6.5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -536,7 +566,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -544,10 +574,13 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -555,22 +588,25 @@
         <v>3</v>
       </c>
       <c r="C5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>32</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>49</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>43</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -578,19 +614,22 @@
         <v>3</v>
       </c>
       <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
         <v>8</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>180</v>
       </c>
-      <c r="F6">
+      <c r="G6">
         <v>80</v>
       </c>
-      <c r="H6" t="s">
+      <c r="I6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -598,16 +637,19 @@
         <v>3</v>
       </c>
       <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
         <v>9</v>
       </c>
-      <c r="G7">
+      <c r="H7">
         <v>250</v>
       </c>
-      <c r="H7" t="s">
+      <c r="I7" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -615,16 +657,19 @@
         <v>3</v>
       </c>
       <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
         <v>10</v>
       </c>
-      <c r="G8">
+      <c r="H8">
         <v>120</v>
       </c>
-      <c r="H8" t="s">
+      <c r="I8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -632,19 +677,22 @@
         <v>3</v>
       </c>
       <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
         <v>11</v>
       </c>
-      <c r="E9">
+      <c r="F9">
         <v>62</v>
       </c>
-      <c r="G9">
+      <c r="H9">
         <v>170</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>14</v>
       </c>
@@ -652,22 +700,25 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s">
         <v>12</v>
       </c>
-      <c r="E10">
+      <c r="F10">
         <v>1</v>
       </c>
-      <c r="F10">
+      <c r="G10">
         <v>4.9000000000000004</v>
       </c>
-      <c r="G10">
+      <c r="H10">
         <v>1.8</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>14</v>
       </c>
@@ -675,6 +726,9 @@
         <v>3</v>
       </c>
       <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>